<commit_message>
docs : update ISMS mapping file with improved version column names
</commit_message>
<xml_diff>
--- a/docs/kisa_isms_p_2023_korean_aws_improved.xlsx
+++ b/docs/kisa_isms_p_2023_korean_aws_improved.xlsx
@@ -46,10 +46,10 @@
     <t>Checks</t>
   </si>
   <si>
-    <t>Purpose(한글)</t>
-  </si>
-  <si>
-    <t>ActionPlan(한글)</t>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>ActionPlan</t>
   </si>
   <si>
     <t>1.1.1</t>

</xml_diff>